<commit_message>
retrieve name by id and total balance
</commit_message>
<xml_diff>
--- a/src/files/tempPDF/etatBoxes.xlsx
+++ b/src/files/tempPDF/etatBoxes.xlsx
@@ -11,34 +11,28 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Édité le : 26/02/2025 à 12:09:33
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>Édité le : 02/03/2025 à 11:58:29
 Par : </t>
   </si>
   <si>
-    <t>État de Caisse des Armateurs</t>
+    <t>État de Caisse d'Armateur : SOFIEN AMICH</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Client</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
+    <t>Caisses vendues</t>
+  </si>
+  <si>
     <t>Caisses récupérées</t>
   </si>
   <si>
-    <t>Caisses vendues</t>
-  </si>
-  <si>
-    <t>SOFIEN AMICH</t>
-  </si>
-  <si>
-    <t>MOHAMED MOHAMED</t>
+    <t>Solde</t>
   </si>
   <si>
     <t>Total</t>
@@ -171,13 +165,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1">
@@ -224,107 +218,85 @@
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="9">
+        <v>45638.75203704</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="9">
+        <v>45695.7625463</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="9">
+        <v>45709.66672454</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="9">
+        <v>45711.67956019</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="9">
-        <v>45638.75203704</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>27</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="5"/>
-      <c r="B7" s="9">
-        <v>45695.7625463</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>80</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="5"/>
-      <c r="B8" s="9">
-        <v>45709.66672454</v>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="5"/>
-      <c r="B9" s="9">
-        <v>45711.67956019</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="9">
-        <v>45638.95833333</v>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>108</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="5"/>
-      <c r="B11" s="9">
-        <v>45689.65009259</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10" t="n">
-        <v>215</v>
-      </c>
-      <c r="D12" s="10" t="n">
-        <v>39</v>
+      <c r="B10" s="10" t="n">
+        <v>107</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>-75</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="B6:B6"/>
-    <mergeCell ref="B7:B7"/>
-    <mergeCell ref="B8:B8"/>
-    <mergeCell ref="B9:B9"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B10:B10"/>
-    <mergeCell ref="B11:B11"/>
-    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A6:A6"/>
+    <mergeCell ref="A7:A7"/>
+    <mergeCell ref="A8:A8"/>
+    <mergeCell ref="A9:A9"/>
+    <mergeCell ref="A10:A10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>